<commit_message>
Starting using real values (persons)
</commit_message>
<xml_diff>
--- a/data/shifts_fixes.xlsx
+++ b/data/shifts_fixes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,103 +424,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Prénom</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Jour</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Début</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fin</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Personne 01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Lundi</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Technique</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>24:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Personne 02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mardi</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Sécurité</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Personne 02</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Vendredi</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sécurité</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>24:00</t>
         </is>
       </c>
     </row>

</xml_diff>